<commit_message>
El Módulo 2 usa la base corregida de la demostración guiada del Módulo 1
La presentación y la descarga Modulo2-Base-Reclamaciones.xlsx pasan a usar
demo-depuracion-datos-SOLUCION.xlsx; se ajustan los ejemplos fijos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Modulo2-Base-Reclamaciones.xlsx
+++ b/Modulo2-Base-Reclamaciones.xlsx
@@ -40,529 +40,529 @@
     <t>Monto Reclamado</t>
   </si>
   <si>
-    <t>REC-3323</t>
-  </si>
-  <si>
-    <t>Nairobi Rosario Rosario</t>
-  </si>
-  <si>
-    <t>002-4782677-4</t>
+    <t>REC-1189</t>
+  </si>
+  <si>
+    <t>Ramón Féliz Jiménez</t>
+  </si>
+  <si>
+    <t>001-4888762-3</t>
   </si>
   <si>
     <t>ARS Humano</t>
   </si>
   <si>
+    <t>Santiago</t>
+  </si>
+  <si>
+    <t>No Registrado</t>
+  </si>
+  <si>
+    <t>Clínica Vista Mar</t>
+  </si>
+  <si>
+    <t>REC-1077</t>
+  </si>
+  <si>
+    <t>Rafael Reyes Gómez</t>
+  </si>
+  <si>
+    <t>047-6491194-0</t>
+  </si>
+  <si>
+    <t>Puerto Plata</t>
+  </si>
+  <si>
+    <t>Hospitalización</t>
+  </si>
+  <si>
+    <t>Centro Médico Las Américas</t>
+  </si>
+  <si>
+    <t>REC-1329</t>
+  </si>
+  <si>
+    <t>María Batista Tavárez</t>
+  </si>
+  <si>
+    <t>001-5317727-3</t>
+  </si>
+  <si>
+    <t>San Cristóbal</t>
+  </si>
+  <si>
+    <t>REC-1280</t>
+  </si>
+  <si>
+    <t>Leidy Ureña Jiménez</t>
+  </si>
+  <si>
+    <t>047-8124028-9</t>
+  </si>
+  <si>
+    <t>Santo Domingo</t>
+  </si>
+  <si>
+    <t>Hospital Regional Norte</t>
+  </si>
+  <si>
+    <t>REC-1168</t>
+  </si>
+  <si>
+    <t>Carmen Guzmán Guzmán</t>
+  </si>
+  <si>
+    <t>031-4969657-9</t>
+  </si>
+  <si>
+    <t>Laboratorio</t>
+  </si>
+  <si>
+    <t>Laboratorio Clínico Amigo</t>
+  </si>
+  <si>
+    <t>REC-1014</t>
+  </si>
+  <si>
+    <t>Miguel Peña Féliz</t>
+  </si>
+  <si>
+    <t>047-9839563-2</t>
+  </si>
+  <si>
     <t>Distrito Nacional</t>
   </si>
   <si>
+    <t>Imágenes</t>
+  </si>
+  <si>
+    <t>REC-1210</t>
+  </si>
+  <si>
+    <t>Julio Díaz Ureña</t>
+  </si>
+  <si>
+    <t>031-4787899-0</t>
+  </si>
+  <si>
+    <t>Emergencia</t>
+  </si>
+  <si>
+    <t>Policlínica Central</t>
+  </si>
+  <si>
+    <t>REC-1140</t>
+  </si>
+  <si>
+    <t>Paola Almonte Almonte</t>
+  </si>
+  <si>
+    <t>047-6491974-2</t>
+  </si>
+  <si>
     <t>Consulta</t>
   </si>
   <si>
+    <t>Centro Médico Nuestra Señora</t>
+  </si>
+  <si>
+    <t>REC-1112</t>
+  </si>
+  <si>
+    <t>Daniela Pérez De la Cruz</t>
+  </si>
+  <si>
+    <t>402-9624033-4</t>
+  </si>
+  <si>
+    <t>REC-1021</t>
+  </si>
+  <si>
+    <t>José Jiménez Ureña</t>
+  </si>
+  <si>
+    <t>037-0045369-6</t>
+  </si>
+  <si>
+    <t>REC-1182</t>
+  </si>
+  <si>
+    <t>Andrés De la Cruz Peña</t>
+  </si>
+  <si>
+    <t>037-5733666-4</t>
+  </si>
+  <si>
+    <t>ARS Universal</t>
+  </si>
+  <si>
+    <t>REC-1056</t>
+  </si>
+  <si>
+    <t>Rosa De la Cruz Rodríguez</t>
+  </si>
+  <si>
+    <t>402-9613027-7</t>
+  </si>
+  <si>
+    <t>REC-1154</t>
+  </si>
+  <si>
+    <t>Marisol Rodríguez Jiménez</t>
+  </si>
+  <si>
+    <t>002-1526365-6</t>
+  </si>
+  <si>
+    <t>La Vega</t>
+  </si>
+  <si>
     <t>Clínica San Rafael</t>
   </si>
   <si>
-    <t>REC-3280</t>
-  </si>
-  <si>
-    <t>Fausto Mercedes Vásquez</t>
-  </si>
-  <si>
-    <t>001-3277401-3</t>
-  </si>
-  <si>
-    <t>La Vega</t>
-  </si>
-  <si>
-    <t>Hospitalización</t>
-  </si>
-  <si>
-    <t>REC-3166</t>
-  </si>
-  <si>
-    <t>Milagros Marte Ogando</t>
-  </si>
-  <si>
-    <t>001-4790390-8</t>
-  </si>
-  <si>
-    <t>San Cristóbal</t>
-  </si>
-  <si>
-    <t>REC-3027</t>
-  </si>
-  <si>
-    <t>Wendy Marte Castillo</t>
-  </si>
-  <si>
-    <t>002-5113435-6</t>
-  </si>
-  <si>
-    <t>Emergencia</t>
-  </si>
-  <si>
-    <t>Laboratorio Clínico Amigo</t>
-  </si>
-  <si>
-    <t>REC-3261</t>
-  </si>
-  <si>
-    <t>Luisa Hernández Polanco</t>
-  </si>
-  <si>
-    <t>402-9199203-0</t>
-  </si>
-  <si>
-    <t>Santiago</t>
-  </si>
-  <si>
-    <t>Policlínica Central</t>
-  </si>
-  <si>
-    <t>REC-3267</t>
-  </si>
-  <si>
-    <t>Bienvenido Castillo Marte</t>
-  </si>
-  <si>
-    <t>001-3772481-5</t>
-  </si>
-  <si>
-    <t>Laboratorio</t>
-  </si>
-  <si>
-    <t>No Registrado</t>
-  </si>
-  <si>
-    <t>REC-3009</t>
-  </si>
-  <si>
-    <t>Héctor Hernández Polanco</t>
-  </si>
-  <si>
-    <t>223-3761950-9</t>
-  </si>
-  <si>
-    <t>Santo Domingo</t>
-  </si>
-  <si>
-    <t>Centro Médico Nuestra Señora</t>
-  </si>
-  <si>
-    <t>REC-3056</t>
-  </si>
-  <si>
-    <t>Fausto Cabrera Hernández</t>
-  </si>
-  <si>
-    <t>031-0856993-9</t>
-  </si>
-  <si>
-    <t>REC-3257</t>
-  </si>
-  <si>
-    <t>Scarlet Polanco Vásquez</t>
-  </si>
-  <si>
-    <t>001-6923102-4</t>
-  </si>
-  <si>
-    <t>Imágenes</t>
-  </si>
-  <si>
-    <t>Clínica Vista Mar</t>
-  </si>
-  <si>
-    <t>REC-3350</t>
-  </si>
-  <si>
-    <t>Dahiana Paulino Hernández</t>
-  </si>
-  <si>
-    <t>001-0168277-4</t>
-  </si>
-  <si>
-    <t>Centro Médico Las Américas</t>
-  </si>
-  <si>
-    <t>REC-3178</t>
-  </si>
-  <si>
-    <t>Domingo Ogando Rosa</t>
-  </si>
-  <si>
-    <t>031-8590736-9</t>
-  </si>
-  <si>
-    <t>REC-3380</t>
-  </si>
-  <si>
-    <t>Dahiana Castillo Sánchez</t>
-  </si>
-  <si>
-    <t>037-2091705-9</t>
-  </si>
-  <si>
-    <t>REC-3138</t>
-  </si>
-  <si>
-    <t>Yesenia Sánchez Paulino</t>
-  </si>
-  <si>
-    <t>031-1735308-6</t>
-  </si>
-  <si>
-    <t>REC-3117</t>
-  </si>
-  <si>
-    <t>Yesenia Castillo Rosario</t>
-  </si>
-  <si>
-    <t>223-8769901-6</t>
-  </si>
-  <si>
-    <t>REC-3115</t>
-  </si>
-  <si>
-    <t>Yokasta Rosa Marte</t>
-  </si>
-  <si>
-    <t>402-6085380-7</t>
-  </si>
-  <si>
-    <t>ARS Universal</t>
-  </si>
-  <si>
-    <t>REC-3154</t>
-  </si>
-  <si>
-    <t>Milagros Rosario Fernández</t>
-  </si>
-  <si>
-    <t>047-8692449-0</t>
-  </si>
-  <si>
-    <t>Puerto Plata</t>
-  </si>
-  <si>
-    <t>REC-3110</t>
-  </si>
-  <si>
-    <t>Alexis Marte Abreu</t>
-  </si>
-  <si>
-    <t>037-8363349-8</t>
-  </si>
-  <si>
-    <t>REC-3186</t>
-  </si>
-  <si>
-    <t>Dahiana Paulino Sánchez</t>
-  </si>
-  <si>
-    <t>402-3178459-7</t>
-  </si>
-  <si>
-    <t>REC-3388</t>
-  </si>
-  <si>
-    <t>Domingo Paulino Beltré</t>
-  </si>
-  <si>
-    <t>002-3426798-5</t>
-  </si>
-  <si>
-    <t>REC-3155</t>
-  </si>
-  <si>
-    <t>Esther Abreu Rosario</t>
-  </si>
-  <si>
-    <t>002-9368611-5</t>
+    <t>REC-1084</t>
+  </si>
+  <si>
+    <t>Wilson Santana Almonte</t>
+  </si>
+  <si>
+    <t>402-8942724-0</t>
   </si>
   <si>
     <t>Centro Diagnóstico del Cibao</t>
   </si>
   <si>
-    <t>REC-3087</t>
-  </si>
-  <si>
-    <t>Fausto Mercedes Hernández</t>
-  </si>
-  <si>
-    <t>001-0379011-0</t>
-  </si>
-  <si>
-    <t>Hospital Regional Norte</t>
-  </si>
-  <si>
-    <t>REC-3116</t>
-  </si>
-  <si>
-    <t>Domingo Hernández Hernández</t>
-  </si>
-  <si>
-    <t>047-8523071-1</t>
-  </si>
-  <si>
-    <t>REC-3095</t>
-  </si>
-  <si>
-    <t>Fausto Fernández Ogando</t>
-  </si>
-  <si>
-    <t>037-4857214-1</t>
-  </si>
-  <si>
-    <t>REC-3231</t>
-  </si>
-  <si>
-    <t>Wilkin Mercedes Fernández</t>
-  </si>
-  <si>
-    <t>002-0656366-0</t>
+    <t>REC-1196</t>
+  </si>
+  <si>
+    <t>Ana Guzmán Mejía</t>
+  </si>
+  <si>
+    <t>402-5600518-8</t>
+  </si>
+  <si>
+    <t>REC-1252</t>
+  </si>
+  <si>
+    <t>Ramón Almonte Batista</t>
+  </si>
+  <si>
+    <t>402-8114714-3</t>
+  </si>
+  <si>
+    <t>REC-1091</t>
+  </si>
+  <si>
+    <t>Rafael Tavárez Díaz</t>
+  </si>
+  <si>
+    <t>037-5381989-8</t>
+  </si>
+  <si>
+    <t>REC-1007</t>
+  </si>
+  <si>
+    <t>Leidy Peña Almonte</t>
+  </si>
+  <si>
+    <t>001-3858598-5</t>
   </si>
   <si>
     <t>MAPFRE Salud ARS</t>
   </si>
   <si>
-    <t>REC-3127</t>
-  </si>
-  <si>
-    <t>Héctor Marte Abreu</t>
-  </si>
-  <si>
-    <t>047-6230304-0</t>
-  </si>
-  <si>
-    <t>REC-3254</t>
-  </si>
-  <si>
-    <t>Bienvenido Sánchez Marte</t>
-  </si>
-  <si>
-    <t>037-6705726-9</t>
-  </si>
-  <si>
-    <t>REC-3214</t>
-  </si>
-  <si>
-    <t>Scarlet Paulino Marte</t>
-  </si>
-  <si>
-    <t>223-6968960-7</t>
-  </si>
-  <si>
-    <t>REC-3188</t>
-  </si>
-  <si>
-    <t>Milagros Paulino Marte</t>
-  </si>
-  <si>
-    <t>402-0725437-6</t>
-  </si>
-  <si>
-    <t>REC-3162</t>
-  </si>
-  <si>
-    <t>Nelson Beltré Cabrera</t>
-  </si>
-  <si>
-    <t>047-3032107-2</t>
-  </si>
-  <si>
-    <t>REC-3365</t>
-  </si>
-  <si>
-    <t>Domingo Hernández Fernández</t>
-  </si>
-  <si>
-    <t>002-4087425-7</t>
-  </si>
-  <si>
-    <t>REC-3106</t>
-  </si>
-  <si>
-    <t>Alexis Rosario Sánchez</t>
-  </si>
-  <si>
-    <t>402-3372244-4</t>
-  </si>
-  <si>
-    <t>REC-3219</t>
-  </si>
-  <si>
-    <t>Rosanna Marte Mercedes</t>
-  </si>
-  <si>
-    <t>402-6023710-3</t>
-  </si>
-  <si>
-    <t>REC-3376</t>
-  </si>
-  <si>
-    <t>Luisa Vásquez Ogando</t>
-  </si>
-  <si>
-    <t>031-5472316-8</t>
+    <t>REC-1042</t>
+  </si>
+  <si>
+    <t>Esperanza Encarnación Pérez</t>
+  </si>
+  <si>
+    <t>002-9497133-3</t>
+  </si>
+  <si>
+    <t>REC-1175</t>
+  </si>
+  <si>
+    <t>Ivelisse Mejía Rosario</t>
+  </si>
+  <si>
+    <t>223-6516549-4</t>
+  </si>
+  <si>
+    <t>REC-1266</t>
+  </si>
+  <si>
+    <t>Mercedes Santana De la Cruz</t>
+  </si>
+  <si>
+    <t>047-9101566-8</t>
+  </si>
+  <si>
+    <t>REC-1336</t>
+  </si>
+  <si>
+    <t>Wilson Pérez De la Cruz</t>
+  </si>
+  <si>
+    <t>002-9024755-8</t>
+  </si>
+  <si>
+    <t>REC-1287</t>
+  </si>
+  <si>
+    <t>Ivelisse Batista Féliz</t>
+  </si>
+  <si>
+    <t>047-0632004-3</t>
+  </si>
+  <si>
+    <t>REC-1161</t>
+  </si>
+  <si>
+    <t>Félix Reyes Peña</t>
+  </si>
+  <si>
+    <t>031-9030576-9</t>
+  </si>
+  <si>
+    <t>REC-1049</t>
+  </si>
+  <si>
+    <t>Yudelka Almonte Martínez</t>
+  </si>
+  <si>
+    <t>002-8951084-0</t>
+  </si>
+  <si>
+    <t>REC-1259</t>
+  </si>
+  <si>
+    <t>Miguel Peña Gómez</t>
+  </si>
+  <si>
+    <t>402-0790644-5</t>
+  </si>
+  <si>
+    <t>REC-1308</t>
+  </si>
+  <si>
+    <t>Ángel Guzmán Reyes</t>
+  </si>
+  <si>
+    <t>002-9145581-4</t>
+  </si>
+  <si>
+    <t>REC-1301</t>
+  </si>
+  <si>
+    <t>María Santana Santana</t>
+  </si>
+  <si>
+    <t>031-1750773-7</t>
+  </si>
+  <si>
+    <t>REC-1231</t>
+  </si>
+  <si>
+    <t>Ivelisse Díaz Batista</t>
+  </si>
+  <si>
+    <t>402-6166805-1</t>
+  </si>
+  <si>
+    <t>REC-1098</t>
+  </si>
+  <si>
+    <t>Carmen Jiménez Castillo</t>
+  </si>
+  <si>
+    <t>223-7547525-4</t>
+  </si>
+  <si>
+    <t>REC-1350</t>
+  </si>
+  <si>
+    <t>Juan Gómez Encarnación</t>
+  </si>
+  <si>
+    <t>001-1338216-9</t>
+  </si>
+  <si>
+    <t>REC-1119</t>
+  </si>
+  <si>
+    <t>Ivelisse Tavárez Pérez</t>
+  </si>
+  <si>
+    <t>037-0451463-1</t>
+  </si>
+  <si>
+    <t>REC-1245</t>
+  </si>
+  <si>
+    <t>Félix Tavárez Cabrera</t>
+  </si>
+  <si>
+    <t>223-0580053-1</t>
+  </si>
+  <si>
+    <t>REC-1028</t>
+  </si>
+  <si>
+    <t>Marisol Díaz Almonte</t>
+  </si>
+  <si>
+    <t>402-7919402-2</t>
   </si>
   <si>
     <t>Primera ARS</t>
   </si>
   <si>
-    <t>REC-3021</t>
-  </si>
-  <si>
-    <t>Mariela Ogando Cabrera</t>
-  </si>
-  <si>
-    <t>223-2032413-6</t>
-  </si>
-  <si>
-    <t>REC-3025</t>
-  </si>
-  <si>
-    <t>Dahiana Castillo Cabrera</t>
-  </si>
-  <si>
-    <t>031-0697598-7</t>
-  </si>
-  <si>
-    <t>REC-3163</t>
-  </si>
-  <si>
-    <t>Wendy Hernández Castillo</t>
-  </si>
-  <si>
-    <t>002-6430100-6</t>
-  </si>
-  <si>
-    <t>REC-3055</t>
-  </si>
-  <si>
-    <t>Mariela Hernández Marte</t>
-  </si>
-  <si>
-    <t>001-0690494-1</t>
-  </si>
-  <si>
-    <t>REC-3134</t>
-  </si>
-  <si>
-    <t>Starling Fernández Hernández</t>
-  </si>
-  <si>
-    <t>402-7803078-1</t>
-  </si>
-  <si>
-    <t>REC-3192</t>
-  </si>
-  <si>
-    <t>Rosanna Paulino Polanco</t>
-  </si>
-  <si>
-    <t>031-4561847-5</t>
-  </si>
-  <si>
-    <t>REC-3004</t>
-  </si>
-  <si>
-    <t>Nelson Sánchez Rosa</t>
-  </si>
-  <si>
-    <t>223-0049162-2</t>
-  </si>
-  <si>
-    <t>REC-3170</t>
-  </si>
-  <si>
-    <t>Nelson Hernández Ogando</t>
-  </si>
-  <si>
-    <t>402-1143947-3</t>
-  </si>
-  <si>
-    <t>REC-3375</t>
-  </si>
-  <si>
-    <t>Scarlet Rosa Hernández</t>
-  </si>
-  <si>
-    <t>031-9878597-5</t>
+    <t>REC-1224</t>
+  </si>
+  <si>
+    <t>Mercedes Guzmán Díaz</t>
+  </si>
+  <si>
+    <t>037-1521978-3</t>
+  </si>
+  <si>
+    <t>REC-1035</t>
+  </si>
+  <si>
+    <t>Rafael Martínez Peña</t>
+  </si>
+  <si>
+    <t>037-2536253-5</t>
+  </si>
+  <si>
+    <t>REC-1105</t>
+  </si>
+  <si>
+    <t>Marisol Ureña Jiménez</t>
+  </si>
+  <si>
+    <t>001-7807309-4</t>
+  </si>
+  <si>
+    <t>REC-1315</t>
+  </si>
+  <si>
+    <t>Mercedes Mejía Féliz</t>
+  </si>
+  <si>
+    <t>002-2527004-8</t>
+  </si>
+  <si>
+    <t>REC-1294</t>
+  </si>
+  <si>
+    <t>Francisco Pérez Núñez</t>
+  </si>
+  <si>
+    <t>223-4138189-9</t>
+  </si>
+  <si>
+    <t>REC-1070</t>
+  </si>
+  <si>
+    <t>Mercedes Guzmán Batista</t>
+  </si>
+  <si>
+    <t>002-6277427-6</t>
+  </si>
+  <si>
+    <t>REC-1126</t>
+  </si>
+  <si>
+    <t>Yudelka Ureña Pérez</t>
+  </si>
+  <si>
+    <t>223-7649596-9</t>
+  </si>
+  <si>
+    <t>REC-1147</t>
+  </si>
+  <si>
+    <t>Rafael Almonte Guzmán</t>
+  </si>
+  <si>
+    <t>031-7828080-0</t>
   </si>
   <si>
     <t>SeNaSa</t>
   </si>
   <si>
-    <t>REC-3111</t>
-  </si>
-  <si>
-    <t>Katherine Sánchez Ogando</t>
-  </si>
-  <si>
-    <t>001-0341912-1</t>
-  </si>
-  <si>
-    <t>REC-3028</t>
-  </si>
-  <si>
-    <t>Eduardo Taveras Polanco</t>
-  </si>
-  <si>
-    <t>037-5458954-0</t>
-  </si>
-  <si>
-    <t>REC-3337</t>
-  </si>
-  <si>
-    <t>Domingo Rosario Ogando</t>
-  </si>
-  <si>
-    <t>031-4509944-5</t>
-  </si>
-  <si>
-    <t>REC-3253</t>
-  </si>
-  <si>
-    <t>Milagros Marte Rosario</t>
-  </si>
-  <si>
-    <t>002-7609778-3</t>
-  </si>
-  <si>
-    <t>REC-3075</t>
-  </si>
-  <si>
-    <t>Yesenia Marte Sánchez</t>
-  </si>
-  <si>
-    <t>223-8248164-2</t>
-  </si>
-  <si>
-    <t>REC-3014</t>
-  </si>
-  <si>
-    <t>Wendy Rosario Cabrera</t>
-  </si>
-  <si>
-    <t>002-8723595-9</t>
-  </si>
-  <si>
-    <t>REC-3175</t>
-  </si>
-  <si>
-    <t>Fausto Castillo Vásquez</t>
-  </si>
-  <si>
-    <t>047-6891328-6</t>
-  </si>
-  <si>
-    <t>REC-3245</t>
-  </si>
-  <si>
-    <t>Luisa Marte Marte</t>
-  </si>
-  <si>
-    <t>037-6237701-5</t>
+    <t>REC-1063</t>
+  </si>
+  <si>
+    <t>Luis Mejía Reyes</t>
+  </si>
+  <si>
+    <t>223-3452548-4</t>
+  </si>
+  <si>
+    <t>REC-1343</t>
+  </si>
+  <si>
+    <t>Altagracia Gómez Núñez</t>
+  </si>
+  <si>
+    <t>047-0784217-6</t>
+  </si>
+  <si>
+    <t>REC-1322</t>
+  </si>
+  <si>
+    <t>Yudelka Féliz Gómez</t>
+  </si>
+  <si>
+    <t>047-8632872-5</t>
+  </si>
+  <si>
+    <t>REC-1273</t>
+  </si>
+  <si>
+    <t>Altagracia Polanco Martínez</t>
+  </si>
+  <si>
+    <t>001-1925992-1</t>
+  </si>
+  <si>
+    <t>REC-1133</t>
+  </si>
+  <si>
+    <t>Julio Tavárez Guzmán</t>
+  </si>
+  <si>
+    <t>001-1614331-5</t>
+  </si>
+  <si>
+    <t>REC-1203</t>
+  </si>
+  <si>
+    <t>Manuel Rodríguez Féliz</t>
+  </si>
+  <si>
+    <t>402-4873161-2</t>
+  </si>
+  <si>
+    <t>REC-1238</t>
+  </si>
+  <si>
+    <t>Ivelisse Ureña Tavárez</t>
+  </si>
+  <si>
+    <t>047-2059000-5</t>
+  </si>
+  <si>
+    <t>REC-1217</t>
+  </si>
+  <si>
+    <t>Carmen Martínez Núñez</t>
+  </si>
+  <si>
+    <t>031-2673256-8</t>
   </si>
 </sst>
 </file>
@@ -1038,10 +1038,10 @@
         <v>15</v>
       </c>
       <c r="H2" s="1">
-        <v>45658</v>
+        <v>45681</v>
       </c>
       <c r="I2" s="2">
-        <v>2989.5</v>
+        <v>12257</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -1064,198 +1064,198 @@
         <v>20</v>
       </c>
       <c r="G3" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="H3" s="1">
-        <v>45670</v>
+        <v>45691</v>
       </c>
       <c r="I3" s="2">
-        <v>140895.5</v>
+        <v>155647</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
         <v>12</v>
       </c>
       <c r="E4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="G4" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="H4" s="1">
-        <v>45681</v>
+        <v>45694</v>
       </c>
       <c r="I4" s="2">
-        <v>2705</v>
+        <v>100732.5</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D5" t="s">
         <v>12</v>
       </c>
       <c r="E5" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="F5" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="G5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H5" s="1">
-        <v>45688</v>
+        <v>45700</v>
       </c>
       <c r="I5" s="2">
-        <v>14111</v>
+        <v>41375</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D6" t="s">
         <v>12</v>
       </c>
       <c r="E6" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="F6" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H6" s="1">
-        <v>45700</v>
+        <v>45710</v>
       </c>
       <c r="I6" s="2">
-        <v>16507.5</v>
+        <v>4768.5</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D7" t="s">
         <v>12</v>
       </c>
       <c r="E7" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="F7" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G7" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="H7" s="1">
-        <v>45704</v>
+        <v>45751</v>
       </c>
       <c r="I7" s="2">
-        <v>4719</v>
+        <v>11332</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C8" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D8" t="s">
         <v>12</v>
       </c>
       <c r="E8" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F8" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="G8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H8" s="1">
-        <v>45714</v>
+        <v>45773</v>
       </c>
       <c r="I8" s="2">
-        <v>3250.5</v>
+        <v>4848.5</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D9" t="s">
         <v>12</v>
       </c>
       <c r="E9" t="s">
-        <v>43</v>
+        <v>13</v>
       </c>
       <c r="F9" t="s">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="G9" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="H9" s="1">
-        <v>45764</v>
+        <v>45794</v>
       </c>
       <c r="I9" s="2">
-        <v>45335.5</v>
+        <v>1880</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B10" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C10" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
@@ -1264,45 +1264,45 @@
         <v>19</v>
       </c>
       <c r="F10" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="G10" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="H10" s="1">
-        <v>45791</v>
+        <v>45805</v>
       </c>
       <c r="I10" s="2">
-        <v>8110</v>
+        <v>11468</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B11" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C11" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D11" t="s">
         <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="F11" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="G11" t="s">
-        <v>56</v>
+        <v>14</v>
       </c>
       <c r="H11" s="1">
-        <v>45794</v>
+        <v>45834</v>
       </c>
       <c r="I11" s="2">
-        <v>3413.5</v>
+        <v>5596.5</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -1316,399 +1316,399 @@
         <v>59</v>
       </c>
       <c r="D12" t="s">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="E12" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="F12" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="G12" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="H12" s="1">
-        <v>45798</v>
+        <v>45692</v>
       </c>
       <c r="I12" s="2">
-        <v>9205.5</v>
+        <v>9809</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>61</v>
+      </c>
+      <c r="B13" t="s">
+        <v>62</v>
+      </c>
+      <c r="C13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" t="s">
         <v>60</v>
       </c>
-      <c r="B13" t="s">
-        <v>61</v>
-      </c>
-      <c r="C13" t="s">
-        <v>62</v>
-      </c>
-      <c r="D13" t="s">
-        <v>12</v>
-      </c>
       <c r="E13" t="s">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="F13" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="G13" t="s">
-        <v>44</v>
+        <v>15</v>
       </c>
       <c r="H13" s="1">
-        <v>45803</v>
+        <v>45732</v>
       </c>
       <c r="I13" s="2">
-        <v>2984.5</v>
+        <v>50257.5</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B14" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C14" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D14" t="s">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="E14" t="s">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="F14" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="G14" t="s">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="H14" s="1">
-        <v>45817</v>
+        <v>45750</v>
       </c>
       <c r="I14" s="2">
-        <v>4301.5</v>
+        <v>12384</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B15" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C15" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D15" t="s">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="E15" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F15" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="G15" t="s">
-        <v>15</v>
+        <v>72</v>
       </c>
       <c r="H15" s="1">
-        <v>45819</v>
+        <v>45758</v>
       </c>
       <c r="I15" s="2">
-        <v>2882.5</v>
+        <v>2793.5</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B16" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C16" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D16" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="E16" t="s">
-        <v>39</v>
+        <v>13</v>
       </c>
       <c r="F16" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="G16" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="H16" s="1">
-        <v>45659</v>
+        <v>45789</v>
       </c>
       <c r="I16" s="2">
-        <v>2333</v>
+        <v>13949</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B17" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C17" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D17" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="E17" t="s">
-        <v>76</v>
+        <v>29</v>
       </c>
       <c r="F17" t="s">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="G17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H17" s="1">
-        <v>45679</v>
+        <v>45805</v>
       </c>
       <c r="I17" s="2">
-        <v>123497</v>
+        <v>3186.5</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B18" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C18" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D18" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="E18" t="s">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="F18" t="s">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="G18" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="H18" s="1">
-        <v>45703</v>
+        <v>45823</v>
       </c>
       <c r="I18" s="2">
-        <v>55375</v>
+        <v>10321</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B19" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C19" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D19" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="E19" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="F19" t="s">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="G19" t="s">
-        <v>56</v>
+        <v>15</v>
       </c>
       <c r="H19" s="1">
-        <v>45706</v>
+        <v>45658</v>
       </c>
       <c r="I19" s="2">
-        <v>150480</v>
+        <v>3158</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B20" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C20" t="s">
+        <v>88</v>
+      </c>
+      <c r="D20" t="s">
         <v>85</v>
       </c>
-      <c r="D20" t="s">
-        <v>72</v>
-      </c>
       <c r="E20" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="F20" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="G20" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="H20" s="1">
-        <v>45735</v>
+        <v>45666</v>
       </c>
       <c r="I20" s="2">
-        <v>3474</v>
+        <v>14587.5</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B21" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C21" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D21" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="E21" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="F21" t="s">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="G21" t="s">
-        <v>89</v>
+        <v>50</v>
       </c>
       <c r="H21" s="1">
-        <v>45785</v>
+        <v>45671</v>
       </c>
       <c r="I21" s="2">
-        <v>16962</v>
+        <v>6107</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B22" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C22" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D22" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="E22" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="F22" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="G22" t="s">
-        <v>93</v>
+        <v>45</v>
       </c>
       <c r="H22" s="1">
-        <v>45789</v>
+        <v>45685</v>
       </c>
       <c r="I22" s="2">
-        <v>13675.5</v>
+        <v>103478</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B23" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C23" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D23" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="E23" t="s">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="F23" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="G23" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H23" s="1">
-        <v>45805</v>
+        <v>45714</v>
       </c>
       <c r="I23" s="2">
-        <v>2314</v>
+        <v>1972</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B24" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C24" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D24" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="E24" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F24" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="G24" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H24" s="1">
-        <v>45830</v>
+        <v>45752</v>
       </c>
       <c r="I24" s="2">
-        <v>4345</v>
+        <v>147899</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B25" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C25" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D25" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="E25" t="s">
-        <v>24</v>
+        <v>67</v>
       </c>
       <c r="F25" t="s">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="G25" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="H25" s="1">
-        <v>45703</v>
+        <v>45759</v>
       </c>
       <c r="I25" s="2">
-        <v>135675.5</v>
+        <v>3309</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -1722,22 +1722,22 @@
         <v>106</v>
       </c>
       <c r="D26" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="E26" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="F26" t="s">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="G26" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="H26" s="1">
-        <v>45723</v>
+        <v>45779</v>
       </c>
       <c r="I26" s="2">
-        <v>6276.5</v>
+        <v>5849.5</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
@@ -1751,22 +1751,22 @@
         <v>109</v>
       </c>
       <c r="D27" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="E27" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="F27" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="G27" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="H27" s="1">
-        <v>45729</v>
+        <v>45790</v>
       </c>
       <c r="I27" s="2">
-        <v>6392.5</v>
+        <v>4638</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -1780,22 +1780,22 @@
         <v>112</v>
       </c>
       <c r="D28" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="E28" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F28" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="G28" t="s">
-        <v>39</v>
+        <v>72</v>
       </c>
       <c r="H28" s="1">
-        <v>45785</v>
+        <v>45796</v>
       </c>
       <c r="I28" s="2">
-        <v>3934</v>
+        <v>3291.5</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
@@ -1809,22 +1809,22 @@
         <v>115</v>
       </c>
       <c r="D29" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="E29" t="s">
-        <v>19</v>
+        <v>67</v>
       </c>
       <c r="F29" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="G29" t="s">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H29" s="1">
-        <v>45798</v>
+        <v>45797</v>
       </c>
       <c r="I29" s="2">
-        <v>2242.5</v>
+        <v>9045</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -1838,22 +1838,22 @@
         <v>118</v>
       </c>
       <c r="D30" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="E30" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="F30" t="s">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="G30" t="s">
-        <v>89</v>
+        <v>50</v>
       </c>
       <c r="H30" s="1">
-        <v>45823</v>
+        <v>45812</v>
       </c>
       <c r="I30" s="2">
-        <v>142937</v>
+        <v>9624.5</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
@@ -1867,22 +1867,22 @@
         <v>121</v>
       </c>
       <c r="D31" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="E31" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F31" t="s">
-        <v>14</v>
+        <v>44</v>
       </c>
       <c r="G31" t="s">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="H31" s="1">
-        <v>45832</v>
+        <v>45821</v>
       </c>
       <c r="I31" s="2">
-        <v>3387</v>
+        <v>16018.5</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -1896,22 +1896,22 @@
         <v>124</v>
       </c>
       <c r="D32" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="E32" t="s">
-        <v>76</v>
+        <v>39</v>
       </c>
       <c r="F32" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="G32" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H32" s="1">
-        <v>45836</v>
+        <v>45822</v>
       </c>
       <c r="I32" s="2">
-        <v>5383</v>
+        <v>1998</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
@@ -1925,22 +1925,22 @@
         <v>127</v>
       </c>
       <c r="D33" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="E33" t="s">
-        <v>24</v>
+        <v>67</v>
       </c>
       <c r="F33" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="G33" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="H33" s="1">
-        <v>45837</v>
+        <v>45826</v>
       </c>
       <c r="I33" s="2">
-        <v>12803</v>
+        <v>118920</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -1954,51 +1954,51 @@
         <v>130</v>
       </c>
       <c r="D34" t="s">
-        <v>131</v>
+        <v>85</v>
       </c>
       <c r="E34" t="s">
-        <v>43</v>
+        <v>13</v>
       </c>
       <c r="F34" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="G34" t="s">
-        <v>56</v>
+        <v>21</v>
       </c>
       <c r="H34" s="1">
-        <v>45687</v>
+        <v>45829</v>
       </c>
       <c r="I34" s="2">
-        <v>13800</v>
+        <v>1357.5</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>131</v>
+      </c>
+      <c r="B35" t="s">
         <v>132</v>
       </c>
-      <c r="B35" t="s">
+      <c r="C35" t="s">
         <v>133</v>
       </c>
-      <c r="C35" t="s">
+      <c r="D35" t="s">
         <v>134</v>
       </c>
-      <c r="D35" t="s">
-        <v>131</v>
-      </c>
       <c r="E35" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="F35" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="G35" t="s">
-        <v>44</v>
+        <v>15</v>
       </c>
       <c r="H35" s="1">
-        <v>45712</v>
+        <v>45658</v>
       </c>
       <c r="I35" s="2">
-        <v>5520</v>
+        <v>1589</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -2012,22 +2012,22 @@
         <v>137</v>
       </c>
       <c r="D36" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="E36" t="s">
-        <v>13</v>
+        <v>39</v>
       </c>
       <c r="F36" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="G36" t="s">
-        <v>89</v>
+        <v>30</v>
       </c>
       <c r="H36" s="1">
-        <v>45720</v>
+        <v>45661</v>
       </c>
       <c r="I36" s="2">
-        <v>9882.5</v>
+        <v>146387.5</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -2041,22 +2041,22 @@
         <v>140</v>
       </c>
       <c r="D37" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="E37" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F37" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="G37" t="s">
-        <v>93</v>
+        <v>21</v>
       </c>
       <c r="H37" s="1">
-        <v>45754</v>
+        <v>45682</v>
       </c>
       <c r="I37" s="2">
-        <v>10122.5</v>
+        <v>129905</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -2070,22 +2070,22 @@
         <v>143</v>
       </c>
       <c r="D38" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="E38" t="s">
-        <v>39</v>
+        <v>67</v>
       </c>
       <c r="F38" t="s">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="G38" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="H38" s="1">
-        <v>45786</v>
+        <v>45692</v>
       </c>
       <c r="I38" s="2">
-        <v>56957.5</v>
+        <v>4224</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -2099,22 +2099,22 @@
         <v>146</v>
       </c>
       <c r="D39" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="E39" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="F39" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="G39" t="s">
         <v>15</v>
       </c>
       <c r="H39" s="1">
-        <v>45818</v>
+        <v>45702</v>
       </c>
       <c r="I39" s="2">
-        <v>11406.5</v>
+        <v>9674.5</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
@@ -2128,22 +2128,22 @@
         <v>149</v>
       </c>
       <c r="D40" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="E40" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F40" t="s">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="G40" t="s">
-        <v>56</v>
+        <v>15</v>
       </c>
       <c r="H40" s="1">
-        <v>45822</v>
+        <v>45712</v>
       </c>
       <c r="I40" s="2">
-        <v>4118.5</v>
+        <v>9291</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
@@ -2157,22 +2157,22 @@
         <v>152</v>
       </c>
       <c r="D41" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="E41" t="s">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="F41" t="s">
         <v>14</v>
       </c>
       <c r="G41" t="s">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="H41" s="1">
-        <v>45823</v>
+        <v>45755</v>
       </c>
       <c r="I41" s="2">
-        <v>2846</v>
+        <v>2675</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
@@ -2186,22 +2186,22 @@
         <v>155</v>
       </c>
       <c r="D42" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="E42" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F42" t="s">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="G42" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="H42" s="1">
-        <v>45827</v>
+        <v>45761</v>
       </c>
       <c r="I42" s="2">
-        <v>9063.5</v>
+        <v>13248</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
@@ -2218,19 +2218,19 @@
         <v>159</v>
       </c>
       <c r="E43" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="F43" t="s">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="G43" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="H43" s="1">
-        <v>45666</v>
+        <v>45684</v>
       </c>
       <c r="I43" s="2">
-        <v>89485</v>
+        <v>4429.5</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
@@ -2247,19 +2247,19 @@
         <v>159</v>
       </c>
       <c r="E44" t="s">
-        <v>43</v>
+        <v>13</v>
       </c>
       <c r="F44" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="G44" t="s">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="H44" s="1">
-        <v>45682</v>
+        <v>45685</v>
       </c>
       <c r="I44" s="2">
-        <v>3211</v>
+        <v>2555</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
@@ -2276,19 +2276,19 @@
         <v>159</v>
       </c>
       <c r="E45" t="s">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="F45" t="s">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="G45" t="s">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="H45" s="1">
-        <v>45719</v>
+        <v>45695</v>
       </c>
       <c r="I45" s="2">
-        <v>10237.5</v>
+        <v>2757.5</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
@@ -2305,19 +2305,19 @@
         <v>159</v>
       </c>
       <c r="E46" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F46" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="G46" t="s">
-        <v>52</v>
+        <v>15</v>
       </c>
       <c r="H46" s="1">
-        <v>45744</v>
+        <v>45704</v>
       </c>
       <c r="I46" s="2">
-        <v>2564</v>
+        <v>14628.5</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -2334,19 +2334,19 @@
         <v>159</v>
       </c>
       <c r="E47" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="F47" t="s">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="G47" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="H47" s="1">
-        <v>45756</v>
+        <v>45715</v>
       </c>
       <c r="I47" s="2">
-        <v>103459.5</v>
+        <v>2013.5</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -2363,19 +2363,19 @@
         <v>159</v>
       </c>
       <c r="E48" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="F48" t="s">
         <v>20</v>
       </c>
       <c r="G48" t="s">
-        <v>93</v>
+        <v>35</v>
       </c>
       <c r="H48" s="1">
-        <v>45759</v>
+        <v>45784</v>
       </c>
       <c r="I48" s="2">
-        <v>117418</v>
+        <v>174865</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
@@ -2392,19 +2392,19 @@
         <v>159</v>
       </c>
       <c r="E49" t="s">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="F49" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G49" t="s">
-        <v>29</v>
+        <v>72</v>
       </c>
       <c r="H49" s="1">
-        <v>45820</v>
+        <v>45790</v>
       </c>
       <c r="I49" s="2">
-        <v>9703.5</v>
+        <v>12998</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
@@ -2421,19 +2421,19 @@
         <v>159</v>
       </c>
       <c r="E50" t="s">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="F50" t="s">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="G50" t="s">
-        <v>93</v>
+        <v>50</v>
       </c>
       <c r="H50" s="1">
-        <v>45820</v>
+        <v>45791</v>
       </c>
       <c r="I50" s="2">
-        <v>11551</v>
+        <v>6390.5</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -2450,19 +2450,19 @@
         <v>159</v>
       </c>
       <c r="E51" t="s">
-        <v>24</v>
+        <v>67</v>
       </c>
       <c r="F51" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="G51" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="H51" s="1">
-        <v>45836</v>
+        <v>45834</v>
       </c>
       <c r="I51" s="2">
-        <v>9542</v>
+        <v>15313</v>
       </c>
     </row>
   </sheetData>

</xml_diff>